<commit_message>
Discount China players in team building (inflated regional stats)
Apply 0.15x multiplier to expected points for China team players when
building teams. China region stats are inflated and don't translate to
international performance. Santiago total improved from 266 to 270 pts,
GW1 jumped from 73 to 108 pts by avoiding China IGLs.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VFL_2026_Santiago_Pricing.xlsx
+++ b/VFL_2026_Santiago_Pricing.xlsx
@@ -2668,70 +2668,70 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>happywei</t>
+          <t>kamo</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Xi Lai Gaming</t>
+          <t>Team Liquid</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>Minny</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDward Gaming</t>
+          <t>Gentle Mates</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>22.3</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+        <v>22</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Minny</t>
+          <t>BABYBAY</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Gentle Mates</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2740,52 +2740,52 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>22.3</v>
+        <v>20.6</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NoMan</t>
+          <t>GLYPH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Xi Lai Gaming</t>
+          <t>Gentle Mates</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0</v>
+        <v>17.7</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GLYPH</t>
+          <t>wayne</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Gentle Mates</t>
+          <t>Team Liquid</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2794,40 +2794,40 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>17.7</v>
+        <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BABYBAY</t>
+          <t>NoMan</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>Xi Lai Gaming</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>20.6</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -2838,13 +2838,13 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>49.5</v>
+        <v>50</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>179.6</v>
+        <v>127.2</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>78</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11">
@@ -2906,12 +2906,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>kamo</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>EDward Gaming</t>
+          <t>Team Liquid</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2920,13 +2920,13 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -2960,81 +2960,81 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GLYPH</t>
+          <t>BABYBAY</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Gentle Mates</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>12.9</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BABYBAY</t>
+          <t>GLYPH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>Gentle Mates</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>12.9</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Xross</t>
+          <t>koalanoob</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Nongshim RedForce</t>
+          <t>FURIA</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
     </row>
@@ -3076,17 +3076,17 @@
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>154.1</v>
+        <v>159.8</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>happywei -&gt; Xross | NoMan -&gt; Lovers rock</t>
+          <t>wayne -&gt; koalanoob | NoMan -&gt; Lovers rock</t>
         </is>
       </c>
     </row>
@@ -3149,27 +3149,27 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>BABYBAY</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>EDward Gaming</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>12.9</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
@@ -3203,12 +3203,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BABYBAY</t>
+          <t>koalanoob</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>FURIA</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3217,52 +3217,52 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>12.9</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Xross</t>
+          <t>Lovers rock</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Nongshim RedForce</t>
+          <t>BBL Esports</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>7.5</v>
+        <v>9.5</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>skuba</t>
+          <t>Ivy</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>Nongshim RedForce</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -3271,46 +3271,46 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Francis</t>
+          <t>invy</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Nongshim RedForce</t>
+          <t>Paper Rex</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>16.7</v>
+        <v>23.7</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
+        <v>35</v>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -3319,17 +3319,17 @@
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>90</v>
+        <v>80.7</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Minny -&gt; skuba | Lovers rock -&gt; Francis</t>
+          <t>Minny -&gt; Ivy | kamo -&gt; invy</t>
         </is>
       </c>
     </row>

</xml_diff>